<commit_message>
docs: reinforce JSON quality rules and add auto-validation in SKILL.md
</commit_message>
<xml_diff>
--- a/skills/doublehit-case-skill/output/TestCases.xlsx
+++ b/skills/doublehit-case-skill/output/TestCases.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J19"/>
+  <dimension ref="A1:J11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -519,12 +519,12 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>自动比价</t>
+          <t>动态表单引擎</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>规则匹配与自动下发</t>
+          <t>基础Schema渲染验证</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -534,21 +534,21 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>SR 属性符合 Active 规则，规则配置为 Auto 模式且价格未超标</t>
+          <t>系统已集成Formily引擎</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>1. 创建满足规则触发条件的 SR
-2. 观察比价引擎运行日志
-3. 检查订单流转状态</t>
+          <t>1. 准备标准元数据JSON
+2. 加载到渲染器
+3. 观察页面表现</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>[UI反馈] 无窗口截断，系统静默处理
-[状态回写] SR 状态更新为 Released to WMS，替换为低价 Carrier
-[审计记录] 记录命中规则 ID 及比价清单</t>
+          <t>[UI反馈] 页面正确渲染对应组件，无白屏
+[状态回写] 状态=ready
+[审计记录] 无需审计</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -567,41 +567,40 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>自动比价</t>
+          <t>元数据驱动</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>API 部分超时跳过逻辑</t>
+          <t>下拉框数据源动态加载</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>异常测试</t>
+          <t>功能测试</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>规则内配置 3 个 Carrier，其中 1 个接口人为制造超时</t>
+          <t>后端API接口正常返回数据</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>1. 触发比价流程
-2. 监控 API 调用链路
-3. 查看最终选中承运商</t>
+          <t>1. 渲染带API URL的下拉组件
+2. 点击下拉列表</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>[UI反馈] 流程不中断，无报错弹窗
-[状态回写] 从成功的 2 个报价中选出最低价并下发
-[审计记录] 记录失败 API 的超时异常日志</t>
+          <t>[UI反馈] 下拉列表展示API返回的选项数据
+[状态回写] 无
+[审计记录] 无需审计</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr"/>
@@ -615,12 +614,12 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>分流决策</t>
+          <t>组件联动</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>报价超标触发人工审核</t>
+          <t>字段显隐被动联动</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -630,25 +629,25 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>价格设置（Price Setting）配置了阈值，SR 报价高于该值</t>
+          <t>Schema配置字段A控制字段B显隐</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>1. 创建 SR 并通过比价获取高额报价
-2. 检查订单列表状态</t>
+          <t>1. 操作字段A满足触发条件
+2. 观察字段B状态</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>[UI反馈] 订单进入 Pending Review 列表
-[状态回写] 状态变更为 Pending Review，截断自动下发
-[审计记录] 记录触发 Pending Review 的原因（报价超标）</t>
+          <t>[UI反馈] 字段B由隐藏转为正常显示
+[状态回写] 字段B.visible=true
+[审计记录] 无需审计</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr"/>
@@ -662,35 +661,35 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>异常保底</t>
+          <t>组件联动</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>API 全失败 Fallback 逻辑</t>
+          <t>字段值更改主动联动</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>边界测试</t>
+          <t>功能测试</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>规则内所有 Carrier 接口均模拟关闭/故障</t>
+          <t>Schema配置字段A更改时主动重置字段C</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>1. 触发比价流程
-2. 观察系统回退动作</t>
+          <t>1. 修改字段A的值
+2. 观察字段C的值</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>[UI反馈] 直接下发，无阻断提示
-[状态回写] 沿用 Original Carrier，状态 Released to WMS
-[审计记录] 记录 API 全失败异常及不卡单回退日志</t>
+          <t>[UI反馈] 字段C内容被自动清空或重置
+[状态回写] 字段C.value=null
+[审计记录] 无需审计</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -709,12 +708,12 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>合并管理</t>
+          <t>数据持久化</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>合并 SR 状态回写一致性</t>
+          <t>业务数据保存接口</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -724,20 +723,20 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>存在多个 Sub-orders 关联至同一合并 SR ID</t>
+          <t>表单填写完毕并校验通过</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>1. 完成合并 SR 的比价与 Carrier 确认
-2. 检查所有关联子单详情</t>
+          <t>1. 点击保存按钮
+2. 检查后端数据库</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>[UI反馈] 列表显示 Carrier 更新成功
-[状态回写] Carrier 及其 Service Level 同步回写至所有关联子单
-[审计记录] 记录合并 SR ID 与子单 ID 的关联变更日志</t>
+          <t>[UI反馈] 提示"保存成功"
+[状态回写] 存储模型新增一条记录
+[审计记录] 无需审计</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -756,40 +755,40 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>人工审核</t>
+          <t>数据持久化</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>手动指定模式互斥交互</t>
+          <t>业务数据回显验证</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>易用性测试</t>
+          <t>功能测试</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>进入 Review 详情页，有系统推荐卡片</t>
+          <t>已存在保存成功的记录ID</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>1. 勾选 Manually specify 复选框
-2. 尝试点击上方的系统建议卡片</t>
+          <t>1. 携带ID刷新页面
+2. 检查表单内容</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>[UI反馈] 上方比价卡片自动变置灰锁定状态，点击无效
-[状态回写] 状态维持 Pending Review
-[审计记录] 记录由系统自动比价转向人工干预的操作</t>
+          <t>[UI反馈] 表单精准还原上次保存的数据
+[状态回写] 加载存储模型对应数据
+[审计记录] 无需审计</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr"/>
@@ -803,34 +802,35 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>人工审核</t>
+          <t>双端校验</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>未选方案点击 Approve 拦截</t>
+          <t>前端正则校验拦截</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>安全测试</t>
+          <t>边界测试</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>进入详情页，取消勾选手动且未点击任何系统卡片</t>
+          <t>字段配置了手机号正则校验</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>1. 尝试点击 Approve &amp; Push 按钮</t>
+          <t>1. 输入非法手机号格式
+2. 点击提交</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>[UI反馈] 按钮置灰或点击弹出警告：“请选择一个激活方案”
-[状态回写] 无状态变更
-[审计记录] 无变更记录</t>
+          <t>[UI反馈] 字段下方红色提示"格式不正确"
+[状态回写] 拦截提交动作
+[审计记录] 无需审计</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -849,40 +849,39 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>人工审核</t>
+          <t>双端校验</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Reject 还原原始方案流水</t>
+          <t>后端校验拦截验证</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>功能测试</t>
+          <t>安全测试</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Pending Review 订单，系统已有推荐低价方案</t>
+          <t>获取保存接口URL</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>1. 点击 Reject 按钮
-2. 在二次确认弹窗选择确定</t>
+          <t>1. 使用Postman绕过前端提交缺失必填项的数据</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>[UI反馈] 弹窗关闭，列表刷新
-[状态回写] 还原为 Original Carrier 并下发至 WMS
-[审计记录] 记录“用户拒绝建议”并回退原始方案的审计信息</t>
+          <t>[UI反馈] 无
+[状态回写] 接口返回400/500错误及规则失败详情
+[审计记录] 无需审计</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr"/>
@@ -896,40 +895,40 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>自动比价</t>
+          <t>动态表单引擎</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>等价价格优先级判定</t>
+          <t>非法Schema容错</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>功能测试</t>
+          <t>异常测试</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>系统中存在两个不同 Carrier 的报价 Total Cost 完全一致</t>
+          <t>Schema接口返回非法JSON字符串</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>1. 触发比价流程
-2. 检查系统默认激发的比价卡片</t>
+          <t>1. 加载非法JSON
+2. 观察页面表现</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>[UI反馈] 自动选中 Carrier Priority 排名靠前的卡片
-[状态回写] 状态 Released to WMS
-[审计记录] 记录因权重降级选中的承运商及顺序</t>
+          <t>[UI反馈] 提示"配置内容加载异常"
+[状态回写] 状态=error
+[审计记录] 无需审计</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr"/>
@@ -943,420 +942,43 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>分流决策</t>
+          <t>异常稳定性</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>多规则满足时锁定优先级最高者</t>
+          <t>并发提交网络抖动</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>功能测试</t>
+          <t>稳定性测试</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>同一个 SR 属性同时满足 A 和 B 两条 Active 规则，A 优先级大于 B</t>
+          <t>高延时网络环境</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>1. 触发 SR 匹配流程
-2. 查看锁定的 Carrier 集合</t>
+          <t>1. 快速点击多次提交按钮</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>[UI反馈] 仅显示规则 A 关联的承运商报价
-[状态回写] 无需人工介入直接流转
-[审计记录] 明确记录锁定规则 A 并停止向下匹配</t>
+          <t>[UI反馈] 第一次点击后按钮置灰，防止重复提交
+[状态回写] 后端仅接收并处理一个请求
+[审计记录] 无需审计</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr"/>
       <c r="J11" s="2" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>TS-CA-011</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>人工审核</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>手动模式获取报价流程</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>功能测试</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>详情页，勾选 Manually specify，已选择 Carrier/Service</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>1. 点击 Request Quote 动作按钮
-2. 观察 Quote Result 区域</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>[UI反馈] Quote Result 区域加载出实时数值并将状态自动置为“激活选中”
-[状态回写] 无状态变更
-[审计记录] 记录手动询价的回执数据（Quote Result）</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="I12" s="2" t="inlineStr"/>
-      <c r="J12" s="2" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>TS-CA-012</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>人工审核</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>Cancel 动作维持原状</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>功能测试</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>订单处于 Pending Review 状态</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>1. 点击审核按钮进入详情
-2. 点击 Cancel 按钮关闭弹窗</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>[UI反馈] 详情弹窗直接关闭
-[状态回写] 订单状态必须保留为 Pending Review，不重置不流转
-[审计记录] 无记录</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="I13" s="2" t="inlineStr"/>
-      <c r="J13" s="2" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>TS-CA-013</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>合并管理</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>合并单属性计算与询价同步</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>边界测试</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>存在 3 个已关联至新 SR ID 的子单，属性分别为不同的重/体积</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>1. 观察合并后 SR 的实物属性汇总值
-2. 对比物流接口收到的 Payload 数据</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>[UI反馈] 详情页汇总属性计算正确
-[状态回写] 暂无
-[审计记录] 记录合并后的总实物属性变更轨迹</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="I14" s="2" t="inlineStr"/>
-      <c r="J14" s="2" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>TS-CA-014</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>人工审核</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>审核详情页数据快照一致性</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>功能测试</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>SR 已进入待审池</t>
-        </is>
-      </c>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>1. 点击 Review 进入详情页
-2. 对比 Summary 模块与列表页/数据库字段值</t>
-        </is>
-      </c>
-      <c r="G15" s="2" t="inlineStr">
-        <is>
-          <t>[UI反馈] 准确展示 Request No.、Warehouse 等 4 个核心字段
-[状态回写] 无
-[审计记录] 系统自动记录审核时的订单基础快照</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="I15" s="2" t="inlineStr"/>
-      <c r="J15" s="2" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>TS-CA-015</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>异常处理</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>手动模式接口超时保底</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>异常测试</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>用户处于手动模式尝试询价，但接口超时</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>1. 点击手动询价按钮并触发超时
-2. 尝试点击 Reject 还原</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="inlineStr">
-        <is>
-          <t>[UI反馈] 系统引导用户使用 Reject 按钮恢复原始方案下发
-[状态回写] 还原 Original Carrier 下发 WMS
-[审计记录] 记录手动询价失败及保底处理路径</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="I16" s="2" t="inlineStr"/>
-      <c r="J16" s="2" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>TS-CA-016</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>分流决策</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>地址无法解析导致保底通行</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>异常测试</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>创建 SR，由于地址字段异常导致无法解析目的地</t>
-        </is>
-      </c>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>1. 触发比价引擎
-2. 检查是否卡单</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="inlineStr">
-        <is>
-          <t>[UI反馈] 判定为路径 C (Fallback)，不卡单下发
-[状态回写] 沿用原始承运商下发 WMS
-[审计记录] 记录因地址解析失败触发不卡单逻辑</t>
-        </is>
-      </c>
-      <c r="H17" s="2" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="I17" s="2" t="inlineStr"/>
-      <c r="J17" s="2" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>TS-CA-017</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>工程安全</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>多用户并发审核冲突校验</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>安全测试</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>两个操作员同时打开同一个 Pending Review 订单的详情</t>
-        </is>
-      </c>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>1. 操作员 A 先行 Approve
-2. 操作员 B 在未刷新的页面点击 Approve</t>
-        </is>
-      </c>
-      <c r="G18" s="2" t="inlineStr">
-        <is>
-          <t>[UI反馈] 操作员 B 收到报错：“订单状态已变更，操作无效”
-[状态回写] 以操作员 A 的提交结果为准
-[审计记录] 拒绝重复写入记录数据</t>
-        </is>
-      </c>
-      <c r="H18" s="2" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="I18" s="2" t="inlineStr"/>
-      <c r="J18" s="2" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>TS-CA-018</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>合并管理</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>子单关联审计完整性</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>安全测试</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t>执行合并询价下发流程</t>
-        </is>
-      </c>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>1. 导出最终审核审计记录
-2. 检查 ID 映射链条</t>
-        </is>
-      </c>
-      <c r="G19" s="2" t="inlineStr">
-        <is>
-          <t>[UI反馈] 暂无
-[状态回写] 子单完成 Carrier 继承同步
-[审计记录] 完整记录初始到最终的全链路审计轨迹</t>
-        </is>
-      </c>
-      <c r="H19" s="2" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="I19" s="2" t="inlineStr"/>
-      <c r="J19" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>